<commit_message>
zh book summary puload excel updated
</commit_message>
<xml_diff>
--- a/audio_ficition/books/excel/book-en.xlsx
+++ b/audio_ficition/books/excel/book-en.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C20"/>
+  <dimension ref="A1:C50"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -448,7 +448,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>0786d048-4a27-4e6c-80a4-a85ca63b4a6e</t>
+          <t>0123742b-5211-4af1-9a4e-1dc134f403d3</t>
         </is>
       </c>
       <c r="B2" t="n">
@@ -456,14 +456,14 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>2025-07-05 17:58:56</t>
+          <t>2025-07-12 12:39:33</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>3cb86557-7add-4b3e-901a-eddf39815438</t>
+          <t>03d19e46-7de6-42b9-9160-f6088b13a1c5</t>
         </is>
       </c>
       <c r="B3" t="n">
@@ -471,14 +471,14 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>2025-06-23 17:58:56</t>
+          <t>2025-07-13 12:39:33</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>400f5353-1dfa-4baa-b9a5-c3c461e3430b</t>
+          <t>0786d048-4a27-4e6c-80a4-a85ca63b4a6e</t>
         </is>
       </c>
       <c r="B4" t="n">
@@ -486,14 +486,14 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>2025-06-24 17:58:56</t>
+          <t>2025-07-05 17:58:56</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>431e6db4-df7a-4523-80f2-7db18fc0763d</t>
+          <t>09459c9e-5d30-4eae-a703-1897b6c45530</t>
         </is>
       </c>
       <c r="B5" t="n">
@@ -501,14 +501,14 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>2025-06-25 17:58:56</t>
+          <t>2025-07-14 12:39:33</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>4323841c-6bd3-406e-b7f5-ac29cb791c1c</t>
+          <t>0abcc181-b239-42d9-8435-63046410e55b</t>
         </is>
       </c>
       <c r="B6" t="n">
@@ -516,14 +516,14 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>2025-06-26 17:58:56</t>
+          <t>2025-07-15 12:39:33</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>4a39abf5-f6bf-4ee3-a1b2-d3d4fb9ee0c1</t>
+          <t>11a93ba3-b264-41c6-9943-3773c81104af</t>
         </is>
       </c>
       <c r="B7" t="n">
@@ -531,14 +531,14 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>2025-07-06 17:58:56</t>
+          <t>2025-07-16 12:39:33</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>4e555ca7-5e1a-4a68-95f3-cacc37a0ba01</t>
+          <t>17187d98-6042-46b9-b2ec-2aabb8d8019f</t>
         </is>
       </c>
       <c r="B8" t="n">
@@ -546,59 +546,47 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>2025-06-27 17:58:56</t>
+          <t>2025-07-17 12:39:33</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>720f6531-bdf2-4c83-9957-0e2c2376d4c0</t>
+          <t>1d279901-9804-4441-9cde-b69bc4f12fe7</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>1</v>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>2025-06-28 17:58:56</t>
-        </is>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="C9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>7befe1c1-be3d-40c3-b57f-606023da546a</t>
+          <t>255e65c1-edba-4a0d-bd5e-46c56edee3dd</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>1</v>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>2025-07-07 17:58:56</t>
-        </is>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="C10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>8419d31b-ab91-4b5b-9871-d4783a800231</t>
+          <t>27d0a303-68c6-464a-bdff-8d19db1d0104</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>1</v>
-      </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>2025-07-08 17:58:56</t>
-        </is>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="C11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>877bd90f-d48e-4985-a335-7d79b3c9228e</t>
+          <t>3cb86557-7add-4b3e-901a-eddf39815438</t>
         </is>
       </c>
       <c r="B12" t="n">
@@ -606,14 +594,14 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>2025-07-09 17:58:56</t>
+          <t>2025-06-23 17:58:56</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>8abf7642-f23d-4da4-a2c9-9d3a062e9460</t>
+          <t>400f5353-1dfa-4baa-b9a5-c3c461e3430b</t>
         </is>
       </c>
       <c r="B13" t="n">
@@ -621,14 +609,14 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>2025-06-29 17:58:56</t>
+          <t>2025-06-24 17:58:56</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>8f9b8311-3892-46d1-bae9-b062e9dcd28f</t>
+          <t>431e6db4-df7a-4523-80f2-7db18fc0763d</t>
         </is>
       </c>
       <c r="B14" t="n">
@@ -636,14 +624,14 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>2025-06-30 17:58:56</t>
+          <t>2025-06-25 17:58:56</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>9aa2e5b4-fe5a-434c-a036-eb6d37c96cbc</t>
+          <t>4323841c-6bd3-406e-b7f5-ac29cb791c1c</t>
         </is>
       </c>
       <c r="B15" t="n">
@@ -651,29 +639,25 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>2025-07-10 17:58:56</t>
+          <t>2025-06-26 17:58:56</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>aaa9a6b2-e054-4eca-86d2-7fed52191e4d</t>
+          <t>4991e7ce-88f6-40b6-97b5-448e7b796209</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>1</v>
-      </c>
-      <c r="C16" t="inlineStr">
-        <is>
-          <t>2025-07-01 17:58:56</t>
-        </is>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="C16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>ad7acc5e-98c0-49a1-a733-d6a362ca2512</t>
+          <t>4a39abf5-f6bf-4ee3-a1b2-d3d4fb9ee0c1</t>
         </is>
       </c>
       <c r="B17" t="n">
@@ -681,14 +665,14 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>2025-07-02 17:58:56</t>
+          <t>2025-07-06 17:58:56</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>b98c82e7-9bf0-4ad0-9fe5-0583956587ce</t>
+          <t>4e555ca7-5e1a-4a68-95f3-cacc37a0ba01</t>
         </is>
       </c>
       <c r="B18" t="n">
@@ -696,14 +680,14 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>2025-07-03 17:58:56</t>
+          <t>2025-06-27 17:58:56</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>be6a7585-9e2f-469f-b037-fdfb1be4c9cf</t>
+          <t>720f6531-bdf2-4c83-9957-0e2c2376d4c0</t>
         </is>
       </c>
       <c r="B19" t="n">
@@ -711,20 +695,390 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>2025-07-04 17:58:56</t>
+          <t>2025-06-28 17:58:56</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
+          <t>7befe1c1-be3d-40c3-b57f-606023da546a</t>
+        </is>
+      </c>
+      <c r="B20" t="n">
+        <v>1</v>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>2025-07-07 17:58:56</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>7d25228b-7032-4a46-b256-6a1fc4eb4b88</t>
+        </is>
+      </c>
+      <c r="B21" t="n">
+        <v>0</v>
+      </c>
+      <c r="C21" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>8419d31b-ab91-4b5b-9871-d4783a800231</t>
+        </is>
+      </c>
+      <c r="B22" t="n">
+        <v>1</v>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>2025-07-08 17:58:56</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>877bd90f-d48e-4985-a335-7d79b3c9228e</t>
+        </is>
+      </c>
+      <c r="B23" t="n">
+        <v>1</v>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>2025-07-09 17:58:56</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>8abf7642-f23d-4da4-a2c9-9d3a062e9460</t>
+        </is>
+      </c>
+      <c r="B24" t="n">
+        <v>1</v>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>2025-06-29 17:58:56</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>8e6c218b-9f33-4a7a-9f7b-cd471a6e194f</t>
+        </is>
+      </c>
+      <c r="B25" t="n">
+        <v>0</v>
+      </c>
+      <c r="C25" t="inlineStr"/>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>8f9b8311-3892-46d1-bae9-b062e9dcd28f</t>
+        </is>
+      </c>
+      <c r="B26" t="n">
+        <v>1</v>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>2025-06-30 17:58:56</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>9aa2e5b4-fe5a-434c-a036-eb6d37c96cbc</t>
+        </is>
+      </c>
+      <c r="B27" t="n">
+        <v>1</v>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>2025-07-10 17:58:56</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>a10b828a-bfba-4837-8582-c7a7ea59a88e</t>
+        </is>
+      </c>
+      <c r="B28" t="n">
+        <v>0</v>
+      </c>
+      <c r="C28" t="inlineStr"/>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>a1767353-8a3b-4936-8e9d-daab48c32bce</t>
+        </is>
+      </c>
+      <c r="B29" t="n">
+        <v>0</v>
+      </c>
+      <c r="C29" t="inlineStr"/>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>a35891e6-6422-4347-8e03-49bbaeb419e1</t>
+        </is>
+      </c>
+      <c r="B30" t="n">
+        <v>0</v>
+      </c>
+      <c r="C30" t="inlineStr"/>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>a3c82621-cb25-49a3-9dad-e3aec327307d</t>
+        </is>
+      </c>
+      <c r="B31" t="n">
+        <v>0</v>
+      </c>
+      <c r="C31" t="inlineStr"/>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>a8773bac-e85a-412b-856f-e28e2a1df706</t>
+        </is>
+      </c>
+      <c r="B32" t="n">
+        <v>0</v>
+      </c>
+      <c r="C32" t="inlineStr"/>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>aaa9a6b2-e054-4eca-86d2-7fed52191e4d</t>
+        </is>
+      </c>
+      <c r="B33" t="n">
+        <v>1</v>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>2025-07-01 17:58:56</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>ab02fc8c-14fd-4406-b846-e6224f4021f5</t>
+        </is>
+      </c>
+      <c r="B34" t="n">
+        <v>0</v>
+      </c>
+      <c r="C34" t="inlineStr"/>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>acc166c0-56c6-4535-8776-8d06f2348d19</t>
+        </is>
+      </c>
+      <c r="B35" t="n">
+        <v>0</v>
+      </c>
+      <c r="C35" t="inlineStr"/>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>ad4db19d-07a6-4d8f-918c-e40511f7c7b9</t>
+        </is>
+      </c>
+      <c r="B36" t="n">
+        <v>0</v>
+      </c>
+      <c r="C36" t="inlineStr"/>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>ad7acc5e-98c0-49a1-a733-d6a362ca2512</t>
+        </is>
+      </c>
+      <c r="B37" t="n">
+        <v>1</v>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>2025-07-02 17:58:56</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>b1036b33-1955-4876-94f3-2775b7dbe0b6</t>
+        </is>
+      </c>
+      <c r="B38" t="n">
+        <v>0</v>
+      </c>
+      <c r="C38" t="inlineStr"/>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>b98c82e7-9bf0-4ad0-9fe5-0583956587ce</t>
+        </is>
+      </c>
+      <c r="B39" t="n">
+        <v>1</v>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>2025-07-03 17:58:56</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>bb506d0f-887e-4f1e-9bc1-9035e92f1baa</t>
+        </is>
+      </c>
+      <c r="B40" t="n">
+        <v>0</v>
+      </c>
+      <c r="C40" t="inlineStr"/>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>be6a7585-9e2f-469f-b037-fdfb1be4c9cf</t>
+        </is>
+      </c>
+      <c r="B41" t="n">
+        <v>1</v>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>2025-07-04 17:58:56</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>c203913f-3f81-40f9-84fa-a8df94efec64</t>
+        </is>
+      </c>
+      <c r="B42" t="n">
+        <v>0</v>
+      </c>
+      <c r="C42" t="inlineStr"/>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>c7caa21c-0a5b-42ab-9ab1-c594a9c4abe3</t>
+        </is>
+      </c>
+      <c r="B43" t="n">
+        <v>0</v>
+      </c>
+      <c r="C43" t="inlineStr"/>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>d257febf-a430-49bd-a0f3-818dcdc2d15d</t>
+        </is>
+      </c>
+      <c r="B44" t="n">
+        <v>0</v>
+      </c>
+      <c r="C44" t="inlineStr"/>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
           <t>d59f7c5e-e4a8-4119-ab2b-24f7e69d7d53</t>
         </is>
       </c>
-      <c r="B20" t="n">
-        <v>1</v>
-      </c>
-      <c r="C20" t="inlineStr"/>
+      <c r="B45" t="n">
+        <v>1</v>
+      </c>
+      <c r="C45" t="inlineStr"/>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>dab1d49d-5a66-4d8b-b261-a6eb1f57b84e</t>
+        </is>
+      </c>
+      <c r="B46" t="n">
+        <v>0</v>
+      </c>
+      <c r="C46" t="inlineStr"/>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>dacd8c9b-772a-4643-a26f-ab2a5fc2ff18</t>
+        </is>
+      </c>
+      <c r="B47" t="n">
+        <v>0</v>
+      </c>
+      <c r="C47" t="inlineStr"/>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>de450e78-5115-464f-8628-72e3a6d9557a</t>
+        </is>
+      </c>
+      <c r="B48" t="n">
+        <v>0</v>
+      </c>
+      <c r="C48" t="inlineStr"/>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>e565156f-b501-44d8-b4c4-acab8359755e</t>
+        </is>
+      </c>
+      <c r="B49" t="n">
+        <v>0</v>
+      </c>
+      <c r="C49" t="inlineStr"/>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>e6a4c96d-aaf3-4b69-ae79-6891fa39f8fc</t>
+        </is>
+      </c>
+      <c r="B50" t="n">
+        <v>0</v>
+      </c>
+      <c r="C50" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>